<commit_message>
chore(data,scripts): remove hardcoded counts and reorder event
- Remove hardcoded `count` fields from books.yaml and notices.yaml
- Update export_books_excel.py to derive count dynamically from book list length
- Reorder Chesapeake commemoration event to chronological position in agenda
- Ensure inventory counts stay synchronized automatically with data changes
</commit_message>
<xml_diff>
--- a/static/documents/SAR_BIBLI_inventaire.xlsx
+++ b/static/documents/SAR_BIBLI_inventaire.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Résumé" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tous les livres" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Biographies" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Marine" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Guerre d'Indépendance Américain" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Histoire Générale" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Lieux Historiques" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Ouvrages Généalogiques" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Répertoires et Relevés" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Sources et Bibliographies" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Catalogues, Colloques, Expos" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Usuels et Revues" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Divers" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Email" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résumé" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tous les livres" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biographies" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marine" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guerre d'Indépendance Américain" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histoire Générale" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lieux Historiques" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ouvrages Généalogiques" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Répertoires et Relevés" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources et Bibliographies" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogues, Colloques, Expos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuels et Revues" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tous les livres'!$A$1:$M$454</definedName>
@@ -7693,7 +7693,7 @@
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>Document généré le 24/03/2026</t>
+          <t>Document généré le 03/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>